<commit_message>
update header of column AP in ssks vorlage
</commit_message>
<xml_diff>
--- a/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/ssks_vorlage.xlsx
+++ b/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/ssks_vorlage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\repos\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EAB46F-80DA-4EB0-A5F6-6F3572689794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154D0876-C95E-4379-A159-438A8BBA7916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="50850" windowHeight="20625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ssks_Beispielbefüllung" sheetId="2" r:id="rId1"/>
@@ -374,11 +374,6 @@
 geordnetes Signal</t>
   </si>
   <si>
-    <t>Weitere
-(z. B. ETCS-Halttafel,
-Vorsignaltafel)</t>
-  </si>
-  <si>
     <t>Dunkel-
 schaltung</t>
   </si>
@@ -386,6 +381,11 @@
     <t>Abstand
 Mastmitte - Gleismitte
 (Gleisabstand)</t>
+  </si>
+  <si>
+    <t>Weitere
+(z. B. ETCS-Halttafel,
+Lf-Signal)</t>
   </si>
 </sst>
 </file>
@@ -1389,7 +1389,7 @@
         <v>108</v>
       </c>
       <c r="K3" s="31" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L3" s="31"/>
       <c r="M3" s="31" t="s">
@@ -1449,13 +1449,13 @@
         <v>66</v>
       </c>
       <c r="AQ3" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="AR3" s="7" t="s">
         <v>103</v>
       </c>
       <c r="AS3" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AT3" s="5" t="s">
         <v>67</v>
@@ -2372,6 +2372,7 @@
     <row r="557" s="16" customFormat="1" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="P3:Q3"/>
     <mergeCell ref="M3:O3"/>
     <mergeCell ref="AW3:AX3"/>
     <mergeCell ref="K3:L3"/>
@@ -2388,7 +2389,6 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="AH3:AN3"/>
     <mergeCell ref="R3:S3"/>
-    <mergeCell ref="P3:Q3"/>
   </mergeCells>
   <pageMargins left="0.78740157480314965" right="0.39370078740157483" top="0.19685039370078741" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
@@ -2400,15 +2400,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E758A0F93049BE4CAD441F10C0D8186D" ma:contentTypeVersion="5" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="fb340e34ecc5d059b634082484788e96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="576ce185-3b2e-4f75-8b7c-efeb82226bea" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae5cd419a40dc0c21009e0c04d2bd83e" ns2:_="" ns3:_="">
     <xsd:import namespace="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
@@ -2600,7 +2591,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -2646,19 +2650,7 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F25B32D-FD26-4105-AE41-4DDE11D43643}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5CD9C34-55B9-46DF-94B7-6C19782F39DF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2677,18 +2669,26 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F25B32D-FD26-4105-AE41-4DDE11D43643}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E76690F-8A23-45F3-AC2B-ADA60E406AB9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5608CC1-62E8-40C3-93D3-D4A0440D7ADA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E76690F-8A23-45F3-AC2B-ADA60E406AB9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Ssks - adjustment of regelzeichnungen (#2481)
* get rid of Ne2 and Ne14 signallings in column AP

* add regelzeichnungen into column R

* update header of column AP in ssks vorlage

* Update table reference

* separate calculation of Regelzeichnung in sskx

---------

Co-authored-by: eclipse-set-bot <set-bot@eclipse.org>
</commit_message>
<xml_diff>
--- a/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/ssks_vorlage.xlsx
+++ b/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/ssks_vorlage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\repos\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EAB46F-80DA-4EB0-A5F6-6F3572689794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154D0876-C95E-4379-A159-438A8BBA7916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="50850" windowHeight="20625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ssks_Beispielbefüllung" sheetId="2" r:id="rId1"/>
@@ -374,11 +374,6 @@
 geordnetes Signal</t>
   </si>
   <si>
-    <t>Weitere
-(z. B. ETCS-Halttafel,
-Vorsignaltafel)</t>
-  </si>
-  <si>
     <t>Dunkel-
 schaltung</t>
   </si>
@@ -386,6 +381,11 @@
     <t>Abstand
 Mastmitte - Gleismitte
 (Gleisabstand)</t>
+  </si>
+  <si>
+    <t>Weitere
+(z. B. ETCS-Halttafel,
+Lf-Signal)</t>
   </si>
 </sst>
 </file>
@@ -1389,7 +1389,7 @@
         <v>108</v>
       </c>
       <c r="K3" s="31" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L3" s="31"/>
       <c r="M3" s="31" t="s">
@@ -1449,13 +1449,13 @@
         <v>66</v>
       </c>
       <c r="AQ3" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="AR3" s="7" t="s">
         <v>103</v>
       </c>
       <c r="AS3" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AT3" s="5" t="s">
         <v>67</v>
@@ -2372,6 +2372,7 @@
     <row r="557" s="16" customFormat="1" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="P3:Q3"/>
     <mergeCell ref="M3:O3"/>
     <mergeCell ref="AW3:AX3"/>
     <mergeCell ref="K3:L3"/>
@@ -2388,7 +2389,6 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="AH3:AN3"/>
     <mergeCell ref="R3:S3"/>
-    <mergeCell ref="P3:Q3"/>
   </mergeCells>
   <pageMargins left="0.78740157480314965" right="0.39370078740157483" top="0.19685039370078741" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
@@ -2400,15 +2400,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E758A0F93049BE4CAD441F10C0D8186D" ma:contentTypeVersion="5" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="fb340e34ecc5d059b634082484788e96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="576ce185-3b2e-4f75-8b7c-efeb82226bea" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae5cd419a40dc0c21009e0c04d2bd83e" ns2:_="" ns3:_="">
     <xsd:import namespace="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
@@ -2600,7 +2591,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -2646,19 +2650,7 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F25B32D-FD26-4105-AE41-4DDE11D43643}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5CD9C34-55B9-46DF-94B7-6C19782F39DF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2677,18 +2669,26 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F25B32D-FD26-4105-AE41-4DDE11D43643}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E76690F-8A23-45F3-AC2B-ADA60E406AB9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5608CC1-62E8-40C3-93D3-D4A0440D7ADA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E76690F-8A23-45F3-AC2B-ADA60E406AB9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Signal Tabelle: update determin side distance (#2570)
* Signal Tabelle: update side distance determine

* Update excel template

* Update table reference

---------

Co-authored-by: eclipse-set-bot <set-bot@eclipse.org>
</commit_message>
<xml_diff>
--- a/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/ssks_vorlage.xlsx
+++ b/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/ssks_vorlage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\repos\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154D0876-C95E-4379-A159-438A8BBA7916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{365524A4-8537-4276-9BE7-895BA1F719BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="50850" windowHeight="20625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ssks_Beispielbefüllung" sheetId="2" r:id="rId1"/>
@@ -378,14 +378,14 @@
 schaltung</t>
   </si>
   <si>
-    <t>Abstand
-Mastmitte - Gleismitte
-(Gleisabstand)</t>
-  </si>
-  <si>
     <t>Weitere
 (z. B. ETCS-Halttafel,
 Lf-Signal)</t>
+  </si>
+  <si>
+    <t>Abstand/Lage
+Mastmitte - Gleismitte
+(Gleisabstand)</t>
   </si>
 </sst>
 </file>
@@ -1389,7 +1389,7 @@
         <v>108</v>
       </c>
       <c r="K3" s="31" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="L3" s="31"/>
       <c r="M3" s="31" t="s">
@@ -1449,7 +1449,7 @@
         <v>66</v>
       </c>
       <c r="AQ3" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="AR3" s="7" t="s">
         <v>103</v>
@@ -2372,6 +2372,7 @@
     <row r="557" s="16" customFormat="1" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="R3:S3"/>
     <mergeCell ref="P3:Q3"/>
     <mergeCell ref="M3:O3"/>
     <mergeCell ref="AW3:AX3"/>
@@ -2388,7 +2389,6 @@
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="AH3:AN3"/>
-    <mergeCell ref="R3:S3"/>
   </mergeCells>
   <pageMargins left="0.78740157480314965" right="0.39370078740157483" top="0.19685039370078741" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
@@ -2400,6 +2400,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E758A0F93049BE4CAD441F10C0D8186D" ma:contentTypeVersion="5" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="fb340e34ecc5d059b634082484788e96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="576ce185-3b2e-4f75-8b7c-efeb82226bea" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae5cd419a40dc0c21009e0c04d2bd83e" ns2:_="" ns3:_="">
     <xsd:import namespace="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
@@ -2591,20 +2600,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -2650,7 +2646,19 @@
 </spe:Receivers>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F25B32D-FD26-4105-AE41-4DDE11D43643}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5CD9C34-55B9-46DF-94B7-6C19782F39DF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2669,26 +2677,18 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F25B32D-FD26-4105-AE41-4DDE11D43643}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5608CC1-62E8-40C3-93D3-D4A0440D7ADA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E76690F-8A23-45F3-AC2B-ADA60E406AB9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5608CC1-62E8-40C3-93D3-D4A0440D7ADA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>